<commit_message>
Amplía cobertura por módulos y documenta ejecución y bloqueos
</commit_message>
<xml_diff>
--- a/entrega/PTP_Juan_Vanegas_23102026.xlsx
+++ b/entrega/PTP_Juan_Vanegas_23102026.xlsx
@@ -2,12 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alcance y estrategia" sheetId="1" r:id="R762106d795ab4967"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP01 Registro" sheetId="2" r:id="R3cfeb4ef9b104a8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP02 Actualizacion" sheetId="3" r:id="R22f3babbd2134658"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP03 Compra" sheetId="4" r:id="Rf28997665e784e4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riesgos y seguimiento" sheetId="5" r:id="Rce7212287efc4a5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repositorio" sheetId="6" r:id="R5583ab570d7d429b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alcance y estrategia" sheetId="1" r:id="R3b569ddd3bc54d51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP01 Registro" sheetId="2" r:id="R9c3d0cb3f6b84d75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP02 Actualizacion" sheetId="3" r:id="R93ab91f81cd34197"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP03 Compra" sheetId="4" r:id="R349f93761bdd4b42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riesgos y seguimiento" sheetId="5" r:id="Rbe132164e66042ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repositorio" sheetId="6" r:id="R195ba0f5c82744b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M1 Zapatos" sheetId="7" r:id="R2b7786c1133949f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M2 Bolsos" sheetId="8" r:id="R49423deedc394827"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M3 Cinturones" sheetId="9" r:id="Rff82be97686e497a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M4 Accesorios" sheetId="10" r:id="R75b83c390d2d4e0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M5 Outlet" sheetId="11" r:id="Re229e50743f04665"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M6 PQRS" sheetId="12" r:id="Rc463606cc4c94c4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M7 Bonos" sheetId="13" r:id="R0e786c957ea045aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M8 Cuenta" sheetId="14" r:id="R1fae8b4525e448ee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +29,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="dd/mm/yyyy"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -64,8 +72,14 @@
       <x:color rgb="FF0563C1"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FF203C67"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -97,6 +111,11 @@
         <x:fgColor rgb="FFEAF0F7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF0F7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -110,7 +129,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="31">
+  <x:cellXfs count="37">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -195,6 +214,20 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -349,13 +382,13 @@
     <xdr:ext cx="9525000" cy="8486775"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="b7ae86d3-c563-4e0b-93cc-918dd108e5b3"/>
+        <xdr:cNvPr id="1" name="/xl/media/image.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R958eba12a34c41f3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5214f4f2dc57423d"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -381,13 +414,13 @@
     <xdr:ext cx="9525000" cy="8486775"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="36f9affd-98c0-4909-b3e9-bfab8fc758d9"/>
+        <xdr:cNvPr id="1" name="/xl/media/image2.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7d8bf8c05d504411"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R665929d4523a4826"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -408,13 +441,13 @@
     <xdr:ext cx="9525000" cy="8658225"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="a9d6ef55-4a37-4cd3-8834-b2628a0c983f"/>
+        <xdr:cNvPr id="2" name="/xl/media/image3.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb0acc9ebb69f4408"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0ce3ab581f69478a"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -697,7 +730,7 @@
         <x:v>Alcance</x:v>
       </x:c>
       <x:c r="C11" s="7" t="str">
-        <x:v>Sitio real: registro y reingreso, modificación y persistencia del nombre, producto/talla/cantidad/subtotal y checkout. La DEMO conserva una confirmación ficticia de compra, separada de los resultados reales.</x:v>
+        <x:v>Tres escenarios principales más ocho pruebas complementarias de catálogos, PQRS, bonos y acceso público. Ver pestañas M1–M8. Compra completa pendiente.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -705,7 +738,7 @@
         <x:v>Fuera de alcance</x:v>
       </x:c>
       <x:c r="C12" s="7" t="str">
-        <x:v>Pagos y pedidos reales, pruebas de carga, seguridad, dispositivos móviles, integraciones internas y automatización exhaustiva de todos los módulos.</x:v>
+        <x:v>Pedidos/pagos reales, radicación PQRS, redención de bonos, carga, seguridad y regresión exhaustiva de todos los módulos.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="54" customHeight="1">
@@ -713,7 +746,7 @@
         <x:v>Priorización</x:v>
       </x:c>
       <x:c r="C13" s="7" t="str">
-        <x:v>Registro y perfil cubren necesidades explícitas. Compra cubre el flujo de ingresos. Los demás módulos quedan como extensión de regresión.</x:v>
+        <x:v>Registro, perfil y compra como escenarios principales. Cobertura adicional por módulo con alcance y resultado medido en cada pestaña M1–M8.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="36" customHeight="1">
@@ -861,6 +894,1107 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="75" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="35" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="35" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="50" customHeight="1">
+      <c r="B2" s="32" t="str">
+        <v>CAT-04 Consultar catálogo y producto de Accesorios</v>
+      </c>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="B5" s="34" t="str">
+        <v>Módulo</v>
+      </c>
+      <c r="C5" s="35" t="str">
+        <v>Accesorios</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="B6" s="34" t="str">
+        <v>Ambiente</v>
+      </c>
+      <c r="C6" s="35" t="str">
+        <v>Bon-Bonite real, sesión pública sin credenciales</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="B7" s="34" t="str">
+        <v>Resultado</v>
+      </c>
+      <c r="C7" s="35" t="str">
+        <v>APROBADO</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" ht="100" customHeight="1">
+      <c r="B8" s="34" t="str">
+        <v>Alcance</v>
+      </c>
+      <c r="C8" s="35" t="str">
+        <v>Seleccionar una ficha desde el catálogo y comprobar nombre, precio numérico e imagen. No certifica filtros, todas las fichas ni compra.</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="B9" s="34" t="str">
+        <v>Código</v>
+      </c>
+      <c r="C9" s="35" t="str">
+        <v>src/test/resources/features/modulos.feature; ModuleSteps.java</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="B10" s="34" t="str">
+        <v>Evidencia</v>
+      </c>
+      <c r="C10" s="36" t="str">
+        <v>Abrir carpeta del reporte complementario</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="B11" s="34" t="str">
+        <v>Ver reporte</v>
+      </c>
+      <c r="C11" s="35" t="str">
+        <v>Descargue GitHub &gt; Code &gt; Download ZIP, descomprima y abra evidencias/Modulos/serenity/index.html.</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="B12" s="34" t="str">
+        <v>Límite</v>
+      </c>
+      <c r="C12" s="35" t="str">
+        <v>Prueba complementaria de la función indicada; no garantiza regresión exhaustiva del módulo.</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="33" t="str">
+        <v>Paso ejecutado</v>
+      </c>
+      <c r="C15" s="33" t="str">
+        <v>Estado medido</v>
+      </c>
+      <c r="D15" s="33" t="str">
+        <v>Descripción</v>
+      </c>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="B16" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="35" t="str">
+        <v>passed</v>
+      </c>
+      <c r="D16" s="35" t="str">
+        <v>que se consulta el catálogo "accesorios-mujer"</v>
+      </c>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="B17" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="35" t="str">
+        <v>passed</v>
+      </c>
+      <c r="D17" s="35" t="str">
+        <v>un producto del catálogo conserva nombre precio e imagen en su ficha</v>
+      </c>
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="B2:E2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence2"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="75" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="35" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="35" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="50" customHeight="1">
+      <c r="B2" s="32" t="str">
+        <v>CAT-05 Consultar catálogo y producto de Outlet</v>
+      </c>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="B5" s="34" t="str">
+        <v>Módulo</v>
+      </c>
+      <c r="C5" s="35" t="str">
+        <v>Outlet</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="B6" s="34" t="str">
+        <v>Ambiente</v>
+      </c>
+      <c r="C6" s="35" t="str">
+        <v>Bon-Bonite real, sesión pública sin credenciales</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="B7" s="34" t="str">
+        <v>Resultado</v>
+      </c>
+      <c r="C7" s="35" t="str">
+        <v>FALLIDO</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" ht="100" customHeight="1">
+      <c r="B8" s="34" t="str">
+        <v>Alcance</v>
+      </c>
+      <c r="C8" s="35" t="str">
+        <v>Seleccionar una ficha desde el catálogo y comprobar nombre, precio numérico e imagen. No certifica filtros, todas las fichas ni compra.</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="B9" s="34" t="str">
+        <v>Código</v>
+      </c>
+      <c r="C9" s="35" t="str">
+        <v>src/test/resources/features/modulos.feature; ModuleSteps.java</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="B10" s="34" t="str">
+        <v>Evidencia</v>
+      </c>
+      <c r="C10" s="36" t="str">
+        <v>Abrir carpeta del reporte complementario</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="B11" s="34" t="str">
+        <v>Ver reporte</v>
+      </c>
+      <c r="C11" s="35" t="str">
+        <v>Descargue GitHub &gt; Code &gt; Download ZIP, descomprima y abra evidencias/Modulos/serenity/index.html.</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="B12" s="34" t="str">
+        <v>Límite</v>
+      </c>
+      <c r="C12" s="35" t="str">
+        <v>Prueba complementaria de la función indicada; no garantiza regresión exhaustiva del módulo.</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="33" t="str">
+        <v>Paso ejecutado</v>
+      </c>
+      <c r="C15" s="33" t="str">
+        <v>Estado medido</v>
+      </c>
+      <c r="D15" s="33" t="str">
+        <v>Descripción</v>
+      </c>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="B16" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="35" t="str">
+        <v>passed</v>
+      </c>
+      <c r="D16" s="35" t="str">
+        <v>que se consulta el catálogo "outlet"</v>
+      </c>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="B17" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="35" t="str">
+        <v>failed</v>
+      </c>
+      <c r="D17" s="35" t="str">
+        <v>un producto del catálogo conserva nombre precio e imagen en su ficha</v>
+      </c>
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="B20" s="35" t="str">
+        <v>Diagnóstico pendiente</v>
+      </c>
+      <c r="C20" s="35" t="str">
+        <v>La ejecución no completó las verificaciones. Se observó 403 Forbidden desde Outlet durante la secuencia. Revisar captura y excepción de este caso en Serenity. No se considera módulo aprobado ni defecto funcional confirmado.</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="B2:E2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence2"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="75" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="35" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="35" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="50" customHeight="1">
+      <c r="B2" s="32" t="str">
+        <v>PQ-01 Correo inválido y opciones de solicitud PQRS</v>
+      </c>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="B5" s="34" t="str">
+        <v>Módulo</v>
+      </c>
+      <c r="C5" s="35" t="str">
+        <v>PQRS</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="B6" s="34" t="str">
+        <v>Ambiente</v>
+      </c>
+      <c r="C6" s="35" t="str">
+        <v>Bon-Bonite real, sesión pública sin credenciales</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="B7" s="34" t="str">
+        <v>Resultado</v>
+      </c>
+      <c r="C7" s="35" t="str">
+        <v>FALLIDO</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" ht="100" customHeight="1">
+      <c r="B8" s="34" t="str">
+        <v>Alcance</v>
+      </c>
+      <c r="C8" s="35" t="str">
+        <v>Opciones de solicitud y validación HTML de correo inválido. No envía PQRS ni certifica radicación.</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="B9" s="34" t="str">
+        <v>Código</v>
+      </c>
+      <c r="C9" s="35" t="str">
+        <v>src/test/resources/features/modulos.feature; ModuleSteps.java</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="B10" s="34" t="str">
+        <v>Evidencia</v>
+      </c>
+      <c r="C10" s="36" t="str">
+        <v>Abrir carpeta del reporte complementario</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="B11" s="34" t="str">
+        <v>Ver reporte</v>
+      </c>
+      <c r="C11" s="35" t="str">
+        <v>Descargue GitHub &gt; Code &gt; Download ZIP, descomprima y abra evidencias/Modulos/serenity/index.html.</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="B12" s="34" t="str">
+        <v>Límite</v>
+      </c>
+      <c r="C12" s="35" t="str">
+        <v>Prueba complementaria de la función indicada; no garantiza regresión exhaustiva del módulo.</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="33" t="str">
+        <v>Paso ejecutado</v>
+      </c>
+      <c r="C15" s="33" t="str">
+        <v>Estado medido</v>
+      </c>
+      <c r="D15" s="33" t="str">
+        <v>Descripción</v>
+      </c>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="B16" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="35" t="str">
+        <v>passed</v>
+      </c>
+      <c r="D16" s="35" t="str">
+        <v>que se consulta PQRS</v>
+      </c>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="B17" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="35" t="str">
+        <v>failed</v>
+      </c>
+      <c r="D17" s="35" t="str">
+        <v>el correo inválido no cumple la validación y existen tipos de solicitud</v>
+      </c>
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="B20" s="35" t="str">
+        <v>Diagnóstico pendiente</v>
+      </c>
+      <c r="C20" s="35" t="str">
+        <v>La ejecución no completó las verificaciones. Se observó 403 Forbidden desde Outlet durante la secuencia. Revisar captura y excepción de este caso en Serenity. No se considera módulo aprobado ni defecto funcional confirmado.</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="B2:E2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence2"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="75" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="35" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="35" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="50" customHeight="1">
+      <c r="B2" s="32" t="str">
+        <v>BO-01 Selección de denominación de bono</v>
+      </c>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="B5" s="34" t="str">
+        <v>Módulo</v>
+      </c>
+      <c r="C5" s="35" t="str">
+        <v>Bonos</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="B6" s="34" t="str">
+        <v>Ambiente</v>
+      </c>
+      <c r="C6" s="35" t="str">
+        <v>Bon-Bonite real, sesión pública sin credenciales</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="B7" s="34" t="str">
+        <v>Resultado</v>
+      </c>
+      <c r="C7" s="35" t="str">
+        <v>FALLIDO</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" ht="100" customHeight="1">
+      <c r="B8" s="34" t="str">
+        <v>Alcance</v>
+      </c>
+      <c r="C8" s="35" t="str">
+        <v>Seleccionar denominación y esperar un identificador de variante. No adquiere ni redime bonos.</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="B9" s="34" t="str">
+        <v>Código</v>
+      </c>
+      <c r="C9" s="35" t="str">
+        <v>src/test/resources/features/modulos.feature; ModuleSteps.java</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="B10" s="34" t="str">
+        <v>Evidencia</v>
+      </c>
+      <c r="C10" s="36" t="str">
+        <v>Abrir carpeta del reporte complementario</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="B11" s="34" t="str">
+        <v>Ver reporte</v>
+      </c>
+      <c r="C11" s="35" t="str">
+        <v>Descargue GitHub &gt; Code &gt; Download ZIP, descomprima y abra evidencias/Modulos/serenity/index.html.</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="B12" s="34" t="str">
+        <v>Límite</v>
+      </c>
+      <c r="C12" s="35" t="str">
+        <v>Prueba complementaria de la función indicada; no garantiza regresión exhaustiva del módulo.</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="33" t="str">
+        <v>Paso ejecutado</v>
+      </c>
+      <c r="C15" s="33" t="str">
+        <v>Estado medido</v>
+      </c>
+      <c r="D15" s="33" t="str">
+        <v>Descripción</v>
+      </c>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="B16" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="35" t="str">
+        <v>passed</v>
+      </c>
+      <c r="D16" s="35" t="str">
+        <v>que se consulta el bono</v>
+      </c>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="B17" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="35" t="str">
+        <v>failed</v>
+      </c>
+      <c r="D17" s="35" t="str">
+        <v>seleccionar una denominación resuelve su variante</v>
+      </c>
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="B20" s="35" t="str">
+        <v>Diagnóstico pendiente</v>
+      </c>
+      <c r="C20" s="35" t="str">
+        <v>La ejecución no completó las verificaciones. Se observó 403 Forbidden desde Outlet durante la secuencia. Revisar captura y excepción de este caso en Serenity. No se considera módulo aprobado ni defecto funcional confirmado.</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="B2:E2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence2"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="75" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="35" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="35" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="50" customHeight="1">
+      <c r="B2" s="32" t="str">
+        <v>AC-01 Acceso y registro Mi cuenta Account</v>
+      </c>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="B5" s="34" t="str">
+        <v>Módulo</v>
+      </c>
+      <c r="C5" s="35" t="str">
+        <v>Cuenta</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="B6" s="34" t="str">
+        <v>Ambiente</v>
+      </c>
+      <c r="C6" s="35" t="str">
+        <v>Bon-Bonite real, sesión pública sin credenciales</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="B7" s="34" t="str">
+        <v>Resultado</v>
+      </c>
+      <c r="C7" s="35" t="str">
+        <v>FALLIDO</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" ht="100" customHeight="1">
+      <c r="B8" s="34" t="str">
+        <v>Alcance</v>
+      </c>
+      <c r="C8" s="35" t="str">
+        <v>Campos de registro, controles obligatorios y tipos de correo/contraseña. Mi cuenta y Account corresponden a la misma ruta; autenticación y perfil están en CP01/CP02.</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="B9" s="34" t="str">
+        <v>Código</v>
+      </c>
+      <c r="C9" s="35" t="str">
+        <v>src/test/resources/features/modulos.feature; ModuleSteps.java</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="B10" s="34" t="str">
+        <v>Evidencia</v>
+      </c>
+      <c r="C10" s="36" t="str">
+        <v>Abrir carpeta del reporte complementario</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="B11" s="34" t="str">
+        <v>Ver reporte</v>
+      </c>
+      <c r="C11" s="35" t="str">
+        <v>Descargue GitHub &gt; Code &gt; Download ZIP, descomprima y abra evidencias/Modulos/serenity/index.html.</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="B12" s="34" t="str">
+        <v>Límite</v>
+      </c>
+      <c r="C12" s="35" t="str">
+        <v>Prueba complementaria de la función indicada; no garantiza regresión exhaustiva del módulo.</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="33" t="str">
+        <v>Paso ejecutado</v>
+      </c>
+      <c r="C15" s="33" t="str">
+        <v>Estado medido</v>
+      </c>
+      <c r="D15" s="33" t="str">
+        <v>Descripción</v>
+      </c>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="B16" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="35" t="str">
+        <v>failed</v>
+      </c>
+      <c r="D16" s="35" t="str">
+        <v>que Juan consulta el formulario público de registro</v>
+      </c>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="B17" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="35" t="str">
+        <v>skipped</v>
+      </c>
+      <c r="D17" s="35" t="str">
+        <v>identifica los campos obligatorios sin enviar datos</v>
+      </c>
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="B20" s="35" t="str">
+        <v>Diagnóstico pendiente</v>
+      </c>
+      <c r="C20" s="35" t="str">
+        <v>La ejecución no completó las verificaciones. Se observó 403 Forbidden desde Outlet durante la secuencia. Revisar captura y excepción de este caso en Serenity. No se considera módulo aprobado ni defecto funcional confirmado.</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="B2:E2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence2"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
@@ -1364,7 +2498,7 @@
     <hyperlink ref="B35" display="Abrir esta captura original en GitHub" tooltip="Abrir esta captura original en GitHub" r:id="rIdEvidence11"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="R3c3b819ba3a5426d"/>
+  <drawing r:id="R10401cbd09884cfc"/>
 </worksheet>
 </file>
 
@@ -2417,7 +3551,7 @@
     <hyperlink ref="B74" display="Abrir esta captura original en GitHub" tooltip="Abrir esta captura original en GitHub" r:id="rIdEvidence14"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="R5850572946fa4b50"/>
+  <drawing r:id="Rdd0455a97ce243b7"/>
 </worksheet>
 </file>
 
@@ -2962,9 +4096,13 @@
         <v>Abrir README: instrucciones para ejecutar y consultar reportes</v>
       </c>
     </row>
-    <row r="24" ht="26" customHeight="1">
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
+    <row r="24" ht="65" customHeight="1">
+      <c r="B24" s="7" t="str">
+        <v>Módulos complementarios</v>
+      </c>
+      <c r="C24" s="7" t="str">
+        <v>Ocho pruebas; ejecutar tools/run.ps1 -Modo Modulos. Reporte: evidencias/Modulos/serenity/index.html. Ver pestañas M1–M8.</v>
+      </c>
     </row>
     <row r="25" ht="26" customHeight="1">
       <c r="B25" s="2"/>
@@ -3007,4 +4145,655 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="75" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="35" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="35" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="50" customHeight="1">
+      <c r="B2" s="32" t="str">
+        <v>CAT-01 Consultar catálogo y producto de Zapatos</v>
+      </c>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="B5" s="34" t="str">
+        <v>Módulo</v>
+      </c>
+      <c r="C5" s="35" t="str">
+        <v>Zapatos</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="B6" s="34" t="str">
+        <v>Ambiente</v>
+      </c>
+      <c r="C6" s="35" t="str">
+        <v>Bon-Bonite real, sesión pública sin credenciales</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="B7" s="34" t="str">
+        <v>Resultado</v>
+      </c>
+      <c r="C7" s="35" t="str">
+        <v>APROBADO</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" ht="100" customHeight="1">
+      <c r="B8" s="34" t="str">
+        <v>Alcance</v>
+      </c>
+      <c r="C8" s="35" t="str">
+        <v>Seleccionar una ficha desde el catálogo y comprobar nombre, precio numérico e imagen. No certifica filtros, todas las fichas ni compra.</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="B9" s="34" t="str">
+        <v>Código</v>
+      </c>
+      <c r="C9" s="35" t="str">
+        <v>src/test/resources/features/modulos.feature; ModuleSteps.java</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="B10" s="34" t="str">
+        <v>Evidencia</v>
+      </c>
+      <c r="C10" s="36" t="str">
+        <v>Abrir carpeta del reporte complementario</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="B11" s="34" t="str">
+        <v>Ver reporte</v>
+      </c>
+      <c r="C11" s="35" t="str">
+        <v>Descargue GitHub &gt; Code &gt; Download ZIP, descomprima y abra evidencias/Modulos/serenity/index.html.</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="B12" s="34" t="str">
+        <v>Límite</v>
+      </c>
+      <c r="C12" s="35" t="str">
+        <v>Prueba complementaria de la función indicada; no garantiza regresión exhaustiva del módulo.</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="33" t="str">
+        <v>Paso ejecutado</v>
+      </c>
+      <c r="C15" s="33" t="str">
+        <v>Estado medido</v>
+      </c>
+      <c r="D15" s="33" t="str">
+        <v>Descripción</v>
+      </c>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="B16" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="35" t="str">
+        <v>passed</v>
+      </c>
+      <c r="D16" s="35" t="str">
+        <v>que se consulta el catálogo "zapatos-mujer"</v>
+      </c>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="B17" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="35" t="str">
+        <v>passed</v>
+      </c>
+      <c r="D17" s="35" t="str">
+        <v>un producto del catálogo conserva nombre precio e imagen en su ficha</v>
+      </c>
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="B2:E2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence2"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="75" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="35" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="35" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="50" customHeight="1">
+      <c r="B2" s="32" t="str">
+        <v>CAT-02 Consultar catálogo y producto de Bolsos</v>
+      </c>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="B5" s="34" t="str">
+        <v>Módulo</v>
+      </c>
+      <c r="C5" s="35" t="str">
+        <v>Bolsos</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="B6" s="34" t="str">
+        <v>Ambiente</v>
+      </c>
+      <c r="C6" s="35" t="str">
+        <v>Bon-Bonite real, sesión pública sin credenciales</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="B7" s="34" t="str">
+        <v>Resultado</v>
+      </c>
+      <c r="C7" s="35" t="str">
+        <v>APROBADO</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" ht="100" customHeight="1">
+      <c r="B8" s="34" t="str">
+        <v>Alcance</v>
+      </c>
+      <c r="C8" s="35" t="str">
+        <v>Seleccionar una ficha desde el catálogo y comprobar nombre, precio numérico e imagen. No certifica filtros, todas las fichas ni compra.</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="B9" s="34" t="str">
+        <v>Código</v>
+      </c>
+      <c r="C9" s="35" t="str">
+        <v>src/test/resources/features/modulos.feature; ModuleSteps.java</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="B10" s="34" t="str">
+        <v>Evidencia</v>
+      </c>
+      <c r="C10" s="36" t="str">
+        <v>Abrir carpeta del reporte complementario</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="B11" s="34" t="str">
+        <v>Ver reporte</v>
+      </c>
+      <c r="C11" s="35" t="str">
+        <v>Descargue GitHub &gt; Code &gt; Download ZIP, descomprima y abra evidencias/Modulos/serenity/index.html.</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="B12" s="34" t="str">
+        <v>Límite</v>
+      </c>
+      <c r="C12" s="35" t="str">
+        <v>Prueba complementaria de la función indicada; no garantiza regresión exhaustiva del módulo.</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="33" t="str">
+        <v>Paso ejecutado</v>
+      </c>
+      <c r="C15" s="33" t="str">
+        <v>Estado medido</v>
+      </c>
+      <c r="D15" s="33" t="str">
+        <v>Descripción</v>
+      </c>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="B16" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="35" t="str">
+        <v>passed</v>
+      </c>
+      <c r="D16" s="35" t="str">
+        <v>que se consulta el catálogo "bolsos-mujer"</v>
+      </c>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="B17" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="35" t="str">
+        <v>passed</v>
+      </c>
+      <c r="D17" s="35" t="str">
+        <v>un producto del catálogo conserva nombre precio e imagen en su ficha</v>
+      </c>
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="B2:E2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence2"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="75" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="35" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="35" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="50" customHeight="1">
+      <c r="B2" s="32" t="str">
+        <v>CAT-03 Consultar catálogo y producto de Cinturones</v>
+      </c>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="B5" s="34" t="str">
+        <v>Módulo</v>
+      </c>
+      <c r="C5" s="35" t="str">
+        <v>Cinturones</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="B6" s="34" t="str">
+        <v>Ambiente</v>
+      </c>
+      <c r="C6" s="35" t="str">
+        <v>Bon-Bonite real, sesión pública sin credenciales</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="B7" s="34" t="str">
+        <v>Resultado</v>
+      </c>
+      <c r="C7" s="35" t="str">
+        <v>APROBADO</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+    </row>
+    <row r="8" ht="100" customHeight="1">
+      <c r="B8" s="34" t="str">
+        <v>Alcance</v>
+      </c>
+      <c r="C8" s="35" t="str">
+        <v>Seleccionar una ficha desde el catálogo y comprobar nombre, precio numérico e imagen. No certifica filtros, todas las fichas ni compra.</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="B9" s="34" t="str">
+        <v>Código</v>
+      </c>
+      <c r="C9" s="35" t="str">
+        <v>src/test/resources/features/modulos.feature; ModuleSteps.java</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="B10" s="34" t="str">
+        <v>Evidencia</v>
+      </c>
+      <c r="C10" s="36" t="str">
+        <v>Abrir carpeta del reporte complementario</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="B11" s="34" t="str">
+        <v>Ver reporte</v>
+      </c>
+      <c r="C11" s="35" t="str">
+        <v>Descargue GitHub &gt; Code &gt; Download ZIP, descomprima y abra evidencias/Modulos/serenity/index.html.</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="B12" s="34" t="str">
+        <v>Límite</v>
+      </c>
+      <c r="C12" s="35" t="str">
+        <v>Prueba complementaria de la función indicada; no garantiza regresión exhaustiva del módulo.</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="33" t="str">
+        <v>Paso ejecutado</v>
+      </c>
+      <c r="C15" s="33" t="str">
+        <v>Estado medido</v>
+      </c>
+      <c r="D15" s="33" t="str">
+        <v>Descripción</v>
+      </c>
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="B16" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="35" t="str">
+        <v>passed</v>
+      </c>
+      <c r="D16" s="35" t="str">
+        <v>que se consulta el catálogo "cinturones-mujer"</v>
+      </c>
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="B17" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="35" t="str">
+        <v>passed</v>
+      </c>
+      <c r="D17" s="35" t="str">
+        <v>un producto del catálogo conserva nombre precio e imagen en su ficha</v>
+      </c>
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="B2:E2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence2"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Revalida cuatro módulos y actualiza resultados aprobados
</commit_message>
<xml_diff>
--- a/entrega/PTP_Juan_Vanegas_23102026.xlsx
+++ b/entrega/PTP_Juan_Vanegas_23102026.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alcance y estrategia" sheetId="1" r:id="R3b569ddd3bc54d51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP01 Registro" sheetId="2" r:id="R9c3d0cb3f6b84d75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP02 Actualizacion" sheetId="3" r:id="R93ab91f81cd34197"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP03 Compra" sheetId="4" r:id="R349f93761bdd4b42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riesgos y seguimiento" sheetId="5" r:id="Rbe132164e66042ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repositorio" sheetId="6" r:id="R195ba0f5c82744b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M1 Zapatos" sheetId="7" r:id="R2b7786c1133949f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M2 Bolsos" sheetId="8" r:id="R49423deedc394827"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M3 Cinturones" sheetId="9" r:id="Rff82be97686e497a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M4 Accesorios" sheetId="10" r:id="R75b83c390d2d4e0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M5 Outlet" sheetId="11" r:id="Re229e50743f04665"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M6 PQRS" sheetId="12" r:id="Rc463606cc4c94c4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M7 Bonos" sheetId="13" r:id="R0e786c957ea045aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M8 Cuenta" sheetId="14" r:id="R1fae8b4525e448ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alcance y estrategia" sheetId="1" r:id="Rb35d3c1777754c29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP01 Registro" sheetId="2" r:id="R80e396582a3e4fa0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP02 Actualizacion" sheetId="3" r:id="R04cf8e8ce0b04d5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CP03 Compra" sheetId="4" r:id="Rd62197276e21400b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riesgos y seguimiento" sheetId="5" r:id="Ra9b27d84b11a4cdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repositorio" sheetId="6" r:id="Rdeb12eeb280d4dbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M1 Zapatos" sheetId="7" r:id="Rc526d965dc8b4526"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M2 Bolsos" sheetId="8" r:id="Rf2cea47bff4b43a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M3 Cinturones" sheetId="9" r:id="Rf11dcb5f7ef74341"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M4 Accesorios" sheetId="10" r:id="Re239c43be739428d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M5 Outlet" sheetId="11" r:id="R2f47450d3229432b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M6 PQRS" sheetId="12" r:id="Rb232e476bb9f4d19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M7 Bonos" sheetId="13" r:id="R3c9b7a77b3384f71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M8 Cuenta" sheetId="14" r:id="Rdf4842309f0e4c2e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -388,7 +388,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5214f4f2dc57423d"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Raa32d7d8e5c44770"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -420,7 +420,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R665929d4523a4826"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8504dfbc7e1f4097"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -447,7 +447,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0ce3ab581f69478a"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R792beab3e1f346fd"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -989,7 +989,7 @@
         <v>Ver reporte</v>
       </c>
       <c r="C11" s="35" t="str">
-        <v>Descargue GitHub &gt; Code &gt; Download ZIP, descomprima y abra evidencias/Modulos/serenity/index.html.</v>
+        <v>Descargue el repositorio y abra evidencias/Modulos/serenity/index.html. M1–M4: primera ejecución; M5–M8: revalidación posterior.</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -1105,7 +1105,7 @@
     <mergeCell ref="B2:E2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence2"/>
+    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1166,7 +1166,7 @@
         <v>Resultado</v>
       </c>
       <c r="C7" s="35" t="str">
-        <v>FALLIDO</v>
+        <v>APROBADO</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1206,7 +1206,7 @@
         <v>Ver reporte</v>
       </c>
       <c r="C11" s="35" t="str">
-        <v>Descargue GitHub &gt; Code &gt; Download ZIP, descomprima y abra evidencias/Modulos/serenity/index.html.</v>
+        <v>Descargue el repositorio y abra evidencias/ModulosRevalidacion/serenity/index.html. M1–M4: primera ejecución; M5–M8: revalidación posterior.</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -1262,7 +1262,7 @@
         <v>2</v>
       </c>
       <c r="C17" s="35" t="str">
-        <v>failed</v>
+        <v>passed</v>
       </c>
       <c r="D17" s="35" t="str">
         <v>un producto del catálogo conserva nombre precio e imagen en su ficha</v>
@@ -1281,13 +1281,9 @@
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
     </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="B20" s="35" t="str">
-        <v>Diagnóstico pendiente</v>
-      </c>
-      <c r="C20" s="35" t="str">
-        <v>La ejecución no completó las verificaciones. Se observó 403 Forbidden desde Outlet durante la secuencia. Revisar captura y excepción de este caso en Serenity. No se considera módulo aprobado ni defecto funcional confirmado.</v>
-      </c>
+    <row r="20">
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
     </row>
@@ -1326,7 +1322,7 @@
     <mergeCell ref="B2:E2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence2"/>
+    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1387,7 +1383,7 @@
         <v>Resultado</v>
       </c>
       <c r="C7" s="35" t="str">
-        <v>FALLIDO</v>
+        <v>APROBADO</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1427,7 +1423,7 @@
         <v>Ver reporte</v>
       </c>
       <c r="C11" s="35" t="str">
-        <v>Descargue GitHub &gt; Code &gt; Download ZIP, descomprima y abra evidencias/Modulos/serenity/index.html.</v>
+        <v>Descargue el repositorio y abra evidencias/ModulosRevalidacion/serenity/index.html. M1–M4: primera ejecución; M5–M8: revalidación posterior.</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -1483,7 +1479,7 @@
         <v>2</v>
       </c>
       <c r="C17" s="35" t="str">
-        <v>failed</v>
+        <v>passed</v>
       </c>
       <c r="D17" s="35" t="str">
         <v>el correo inválido no cumple la validación y existen tipos de solicitud</v>
@@ -1502,13 +1498,9 @@
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
     </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="B20" s="35" t="str">
-        <v>Diagnóstico pendiente</v>
-      </c>
-      <c r="C20" s="35" t="str">
-        <v>La ejecución no completó las verificaciones. Se observó 403 Forbidden desde Outlet durante la secuencia. Revisar captura y excepción de este caso en Serenity. No se considera módulo aprobado ni defecto funcional confirmado.</v>
-      </c>
+    <row r="20">
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
     </row>
@@ -1547,7 +1539,7 @@
     <mergeCell ref="B2:E2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence2"/>
+    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1608,7 +1600,7 @@
         <v>Resultado</v>
       </c>
       <c r="C7" s="35" t="str">
-        <v>FALLIDO</v>
+        <v>APROBADO</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1648,7 +1640,7 @@
         <v>Ver reporte</v>
       </c>
       <c r="C11" s="35" t="str">
-        <v>Descargue GitHub &gt; Code &gt; Download ZIP, descomprima y abra evidencias/Modulos/serenity/index.html.</v>
+        <v>Descargue el repositorio y abra evidencias/ModulosRevalidacion/serenity/index.html. M1–M4: primera ejecución; M5–M8: revalidación posterior.</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -1704,7 +1696,7 @@
         <v>2</v>
       </c>
       <c r="C17" s="35" t="str">
-        <v>failed</v>
+        <v>passed</v>
       </c>
       <c r="D17" s="35" t="str">
         <v>seleccionar una denominación resuelve su variante</v>
@@ -1723,13 +1715,9 @@
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
     </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="B20" s="35" t="str">
-        <v>Diagnóstico pendiente</v>
-      </c>
-      <c r="C20" s="35" t="str">
-        <v>La ejecución no completó las verificaciones. Se observó 403 Forbidden desde Outlet durante la secuencia. Revisar captura y excepción de este caso en Serenity. No se considera módulo aprobado ni defecto funcional confirmado.</v>
-      </c>
+    <row r="20">
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
     </row>
@@ -1768,7 +1756,7 @@
     <mergeCell ref="B2:E2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence2"/>
+    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1829,7 +1817,7 @@
         <v>Resultado</v>
       </c>
       <c r="C7" s="35" t="str">
-        <v>FALLIDO</v>
+        <v>APROBADO</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1869,7 +1857,7 @@
         <v>Ver reporte</v>
       </c>
       <c r="C11" s="35" t="str">
-        <v>Descargue GitHub &gt; Code &gt; Download ZIP, descomprima y abra evidencias/Modulos/serenity/index.html.</v>
+        <v>Descargue el repositorio y abra evidencias/ModulosRevalidacion/serenity/index.html. M1–M4: primera ejecución; M5–M8: revalidación posterior.</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -1913,7 +1901,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="35" t="str">
-        <v>failed</v>
+        <v>passed</v>
       </c>
       <c r="D16" s="35" t="str">
         <v>que Juan consulta el formulario público de registro</v>
@@ -1925,7 +1913,7 @@
         <v>2</v>
       </c>
       <c r="C17" s="35" t="str">
-        <v>skipped</v>
+        <v>passed</v>
       </c>
       <c r="D17" s="35" t="str">
         <v>identifica los campos obligatorios sin enviar datos</v>
@@ -1944,13 +1932,9 @@
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
     </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="B20" s="35" t="str">
-        <v>Diagnóstico pendiente</v>
-      </c>
-      <c r="C20" s="35" t="str">
-        <v>La ejecución no completó las verificaciones. Se observó 403 Forbidden desde Outlet durante la secuencia. Revisar captura y excepción de este caso en Serenity. No se considera módulo aprobado ni defecto funcional confirmado.</v>
-      </c>
+    <row r="20">
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
     </row>
@@ -1989,7 +1973,7 @@
     <mergeCell ref="B2:E2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence2"/>
+    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2498,7 +2482,7 @@
     <hyperlink ref="B35" display="Abrir esta captura original en GitHub" tooltip="Abrir esta captura original en GitHub" r:id="rIdEvidence11"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="R10401cbd09884cfc"/>
+  <drawing r:id="R27c1fbf26e8f4807"/>
 </worksheet>
 </file>
 
@@ -3551,7 +3535,7 @@
     <hyperlink ref="B74" display="Abrir esta captura original en GitHub" tooltip="Abrir esta captura original en GitHub" r:id="rIdEvidence14"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="Rdd0455a97ce243b7"/>
+  <drawing r:id="Rd90021bea84744cf"/>
 </worksheet>
 </file>
 
@@ -4242,7 +4226,7 @@
         <v>Ver reporte</v>
       </c>
       <c r="C11" s="35" t="str">
-        <v>Descargue GitHub &gt; Code &gt; Download ZIP, descomprima y abra evidencias/Modulos/serenity/index.html.</v>
+        <v>Descargue el repositorio y abra evidencias/Modulos/serenity/index.html. M1–M4: primera ejecución; M5–M8: revalidación posterior.</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -4358,7 +4342,7 @@
     <mergeCell ref="B2:E2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence2"/>
+    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4459,7 +4443,7 @@
         <v>Ver reporte</v>
       </c>
       <c r="C11" s="35" t="str">
-        <v>Descargue GitHub &gt; Code &gt; Download ZIP, descomprima y abra evidencias/Modulos/serenity/index.html.</v>
+        <v>Descargue el repositorio y abra evidencias/Modulos/serenity/index.html. M1–M4: primera ejecución; M5–M8: revalidación posterior.</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -4575,7 +4559,7 @@
     <mergeCell ref="B2:E2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence2"/>
+    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4676,7 +4660,7 @@
         <v>Ver reporte</v>
       </c>
       <c r="C11" s="35" t="str">
-        <v>Descargue GitHub &gt; Code &gt; Download ZIP, descomprima y abra evidencias/Modulos/serenity/index.html.</v>
+        <v>Descargue el repositorio y abra evidencias/Modulos/serenity/index.html. M1–M4: primera ejecución; M5–M8: revalidación posterior.</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -4792,7 +4776,7 @@
     <mergeCell ref="B2:E2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence2"/>
+    <hyperlink ref="C10" display="Abrir carpeta del reporte complementario" tooltip="Abrir carpeta del reporte complementario" r:id="rIdEvidence1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>